<commit_message>
Updated code for Sloveakia JobChanges script and added JobChangePage.
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Slovakia_Regression_PK17.xlsx
+++ b/Data/Hires/Workday_NewHire_Slovakia_Regression_PK17.xlsx
@@ -1,20 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{4715BC09-F8B0-4900-88B1-1DD6DAA1149E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7360"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="131">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -235,24 +250,12 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10699090</t>
-  </si>
-  <si>
-    <t>Passed</t>
-  </si>
-  <si>
     <t>870 Recruitment (Wazup Zudimi (9581610))</t>
   </si>
   <si>
     <t>Slovakia</t>
   </si>
   <si>
-    <t>Einar</t>
-  </si>
-  <si>
-    <t>Metz</t>
-  </si>
-  <si>
     <t>041/562 66 84</t>
   </si>
   <si>
@@ -319,7 +322,7 @@
     <t>SK Monthly</t>
   </si>
   <si>
-    <t xml:space="preserve">Meal Voucher Card </t>
+    <t>Meal Voucher Card </t>
   </si>
   <si>
     <t>Všeobecná zdrav. Poisť.</t>
@@ -383,19 +386,10 @@
     <t>Test2</t>
   </si>
   <si>
-    <t>10699091</t>
-  </si>
-  <si>
     <t>870 Store Management (Wazup Zudimi (9581610))</t>
   </si>
   <si>
-    <t>Werner</t>
-  </si>
-  <si>
-    <t>Welch</t>
-  </si>
-  <si>
-    <t>Auto 90126088</t>
+    <t>Auto 30165015</t>
   </si>
   <si>
     <t>Permanent</t>
@@ -423,51 +417,57 @@
   </si>
   <si>
     <t>Female</t>
+  </si>
+  <si>
+    <t>Auto 89024414</t>
+  </si>
+  <si>
+    <t>Auto 19951165</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <color rgb="FFFF0000"/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -476,18 +476,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.5999938962981048"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -507,17 +513,27 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -527,15 +543,25 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -546,7 +572,9 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -556,38 +584,56 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -694,6 +740,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -975,9 +1027,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:CH3"/>
-  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:CH7"/>
+  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="10.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" style="1" customWidth="1"/>
@@ -1067,7 +1119,7 @@
     <col min="87" max="87" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.5" customHeight="1" spans="1:86" s="3" customFormat="1" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="1" spans="1:86" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1305,45 +1357,37 @@
       <c r="CG1" s="11"/>
       <c r="CH1" s="12"/>
     </row>
-    <row r="2" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="36"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" s="14" t="s">
+      <c r="E2" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="16"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="I2" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="J2" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="G2" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="H2" s="15" t="s">
+      <c r="K2" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="L2" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="M2" s="18" t="s">
         <v>79</v>
-      </c>
-      <c r="I2" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="J2" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="K2" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="M2" s="18" t="s">
-        <v>83</v>
       </c>
       <c r="N2" s="18">
         <v>1</v>
@@ -1355,188 +1399,188 @@
         <v>90851</v>
       </c>
       <c r="Q2" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="R2" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="S2" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="T2" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="U2" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="V2" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="W2" s="21">
+        <f t="shared" ref="W2:W7" ca="1" si="0">TODAY()-31</f>
+        <v>45794</v>
+      </c>
+      <c r="X2" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y2" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="R2" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="S2" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="T2" s="19" t="s">
+      <c r="Z2" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="U2" s="20" t="s">
+      <c r="AA2" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="V2" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="W2" s="21">
-        <f t="shared" ref="W2:W3" si="0">TODAY()-31</f>
-        <v>45761</v>
-      </c>
-      <c r="X2" s="18" t="s">
+      <c r="AB2" s="19" t="s">
         <v>87</v>
-      </c>
-      <c r="Y2" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="Z2" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="AA2" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="AB2" s="19" t="s">
-        <v>91</v>
       </c>
       <c r="AC2" s="15">
         <v>870</v>
       </c>
       <c r="AD2" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE2" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="AF2" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG2" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH2" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI2" s="21">
+        <f ca="1">TODAY()+365</f>
+        <v>46190</v>
+      </c>
+      <c r="AJ2" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="AE2" s="15" t="s">
+      <c r="AK2" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="AF2" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="AG2" s="15" t="s">
+      <c r="AL2" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="AH2" s="15" t="s">
+      <c r="AM2" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="AI2" s="21">
-        <f>TODAY()+365</f>
-        <v>46157</v>
-      </c>
-      <c r="AJ2" s="18" t="s">
+      <c r="AN2" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="AK2" s="25" t="s">
+      <c r="AO2" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="AL2" s="25" t="s">
+      <c r="AP2" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="AM2" s="18" t="s">
+      <c r="AQ2" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AR2" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS2" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AT2" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU2" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV2" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="AN2" s="18" t="s">
+      <c r="AW2" s="26" t="s">
         <v>100</v>
-      </c>
-      <c r="AO2" s="24" t="s">
-        <v>101</v>
-      </c>
-      <c r="AP2" s="26" t="s">
-        <v>102</v>
-      </c>
-      <c r="AQ2" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="AR2" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="AS2" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="AT2" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="AU2" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="AV2" s="26" t="s">
-        <v>103</v>
-      </c>
-      <c r="AW2" s="26" t="s">
-        <v>104</v>
       </c>
       <c r="AX2" s="27">
         <v>1234567891</v>
       </c>
       <c r="AY2" s="15" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="AZ2" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="BA2" s="19">
+        <f t="shared" ref="BA2:BA7" ca="1" si="1">TODAY()+90</f>
+        <v>45915</v>
+      </c>
+      <c r="BB2" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="BC2" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="BD2" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="BE2" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="BA2" s="19">
-        <f t="shared" ref="BA2:BA3" si="1">TODAY()+90</f>
-        <v>45882</v>
-      </c>
-      <c r="BB2" s="15" t="s">
+      <c r="BF2" s="19">
+        <f t="shared" ref="BF2:BF3" ca="1" si="2">W2</f>
+        <v>45794</v>
+      </c>
+      <c r="BG2" s="19">
+        <f t="shared" ref="BG2:BG3" ca="1" si="3">W2</f>
+        <v>45794</v>
+      </c>
+      <c r="BH2" s="21">
+        <f t="shared" ref="BH2:BH3" ca="1" si="4">AI2</f>
+        <v>46190</v>
+      </c>
+      <c r="BI2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BJ2" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="BC2" s="18" t="s">
+      <c r="BK2" s="30">
+        <f t="array" aca="1" ref="BK2:BK3" ca="1">_xlfn.RANDARRAY(2,1,123456789,999999999,TRUE)</f>
+        <v>571268906</v>
+      </c>
+      <c r="BL2" s="31" t="s">
         <v>107</v>
       </c>
-      <c r="BD2" s="15" t="s">
+      <c r="BM2" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="BE2" s="18" t="s">
+      <c r="BN2" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="BF2" s="19">
-        <f t="shared" ref="BF2:BF3" si="2">W2</f>
-        <v>45761</v>
-      </c>
-      <c r="BG2" s="19">
-        <f t="shared" ref="BG2:BG3" si="3">W2</f>
-        <v>45761</v>
-      </c>
-      <c r="BH2" s="21">
-        <f t="shared" ref="BH2:BH3" si="4">AI2</f>
-        <v>46157</v>
-      </c>
-      <c r="BI2" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="BJ2" s="29" t="s">
+      <c r="BO2" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="BK2" s="30">
-        <f t="array" ref="BK2:BK3">_xlfn.RANDARRAY(2,1,123456789,999999999,TRUE)</f>
-        <v>497291593</v>
-      </c>
-      <c r="BL2" s="31" t="s">
+      <c r="BP2" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="BQ2" s="28" t="s">
         <v>111</v>
       </c>
-      <c r="BM2" s="19" t="s">
+      <c r="BR2" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BS2" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="BN2" s="28" t="s">
+      <c r="BT2" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="BO2" s="28" t="s">
+      <c r="BU2" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="BP2" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="BQ2" s="28" t="s">
+      <c r="BV2" s="28" t="s">
         <v>115</v>
       </c>
-      <c r="BR2" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="BS2" s="15" t="s">
+      <c r="BW2" s="28" t="s">
         <v>116</v>
-      </c>
-      <c r="BT2" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="BU2" s="28" t="s">
-        <v>118</v>
-      </c>
-      <c r="BV2" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="BW2" s="28" t="s">
-        <v>120</v>
       </c>
       <c r="BX2" s="33"/>
       <c r="BY2" s="33"/>
@@ -1550,45 +1594,37 @@
       <c r="CG2" s="33"/>
       <c r="CH2" s="33"/>
     </row>
-    <row r="3" ht="15.65" customHeight="1" spans="1:86" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="35" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>74</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="B3" s="37"/>
+      <c r="C3" s="13"/>
       <c r="D3" s="14" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E3" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="16"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="I3" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F3" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="G3" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="H3" s="15" t="s">
+      <c r="J3" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="M3" s="18" t="s">
         <v>79</v>
-      </c>
-      <c r="I3" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="J3" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="K3" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="L3" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="M3" s="18" t="s">
-        <v>83</v>
       </c>
       <c r="N3" s="18">
         <v>1</v>
@@ -1600,47 +1636,47 @@
         <v>90851</v>
       </c>
       <c r="Q3" s="18" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="R3" s="18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="S3" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="T3" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="T3" s="19" t="s">
-        <v>85</v>
-      </c>
       <c r="U3" s="20" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="V3" s="18" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="W3" s="21">
-        <f t="shared" si="0"/>
-        <v>45761</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45794</v>
       </c>
       <c r="X3" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y3" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="Z3" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA3" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="AB3" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="Y3" s="22" t="s">
-        <v>126</v>
-      </c>
-      <c r="Z3" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA3" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="AB3" s="19" t="s">
-        <v>91</v>
-      </c>
       <c r="AC3" s="15" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="AD3" s="15" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="AE3" s="15">
         <v>40</v>
@@ -1649,137 +1685,138 @@
         <v>40</v>
       </c>
       <c r="AG3" s="15" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AH3" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI3" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="AJ3" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="AK3" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="AL3" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="AM3" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="AI3" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="AJ3" s="18" t="s">
+      <c r="AN3" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="AK3" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="AL3" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="AM3" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="AN3" s="18" t="s">
-        <v>100</v>
-      </c>
       <c r="AO3" s="24" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="AP3" s="26" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="AQ3" s="15" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="AR3" s="19" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AS3" s="15" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="AT3" s="19" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AU3" s="19" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AV3" s="26" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AW3" s="26" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AX3" s="26" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AY3" s="15" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="AZ3" s="21" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="BA3" s="19">
-        <f t="shared" si="1"/>
-        <v>45882</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45915</v>
       </c>
       <c r="BB3" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="BC3" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="BD3" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="BE3" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="BF3" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>45794</v>
+      </c>
+      <c r="BG3" s="19">
+        <f t="shared" ca="1" si="3"/>
+        <v>45794</v>
+      </c>
+      <c r="BH3" s="21" t="str">
+        <f t="shared" si="4"/>
+        <v>N/A</v>
+      </c>
+      <c r="BI3" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BJ3" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="BC3" s="18" t="s">
-        <v>107</v>
-      </c>
-      <c r="BD3" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="BE3" s="18" t="s">
+      <c r="BK3" s="30">
+        <f ca="1"/>
+        <v>427497548</v>
+      </c>
+      <c r="BL3" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM3" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="BN3" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="BF3" s="19">
-        <f t="shared" si="2"/>
-        <v>45761</v>
-      </c>
-      <c r="BG3" s="19">
-        <f t="shared" si="3"/>
-        <v>45761</v>
-      </c>
-      <c r="BH3" s="21">
-        <f t="shared" si="4"/>
-        <v>NaN</v>
-      </c>
-      <c r="BI3" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="BJ3" s="29" t="s">
+      <c r="BO3" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="BK3" s="30">
-        <v>392642536</v>
-      </c>
-      <c r="BL3" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="BM3" s="19" t="s">
+      <c r="BP3" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="BQ3" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="BR3" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BS3" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="BN3" s="28" t="s">
+      <c r="BT3" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="BO3" s="28" t="s">
+      <c r="BU3" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="BP3" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="BQ3" s="28" t="s">
+      <c r="BV3" s="28" t="s">
         <v>115</v>
       </c>
-      <c r="BR3" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="BS3" s="15" t="s">
+      <c r="BW3" s="28" t="s">
         <v>116</v>
-      </c>
-      <c r="BT3" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="BU3" s="28" t="s">
-        <v>118</v>
-      </c>
-      <c r="BV3" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="BW3" s="28" t="s">
-        <v>120</v>
       </c>
       <c r="BX3" s="33"/>
       <c r="BY3" s="33"/>
@@ -1793,36 +1830,968 @@
       <c r="CG3" s="33"/>
       <c r="CH3" s="33"/>
     </row>
+    <row r="4" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="36"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" s="16"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="J4" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="K4" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="L4" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="M4" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="N4" s="18">
+        <v>1</v>
+      </c>
+      <c r="O4" s="18">
+        <v>1612</v>
+      </c>
+      <c r="P4" s="18">
+        <v>90851</v>
+      </c>
+      <c r="Q4" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="R4" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="S4" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="T4" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="U4" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="V4" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="W4" s="21">
+        <f t="shared" ca="1" si="0"/>
+        <v>45794</v>
+      </c>
+      <c r="X4" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y4" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="Z4" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA4" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="AB4" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC4" s="15">
+        <v>870</v>
+      </c>
+      <c r="AD4" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE4" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="AF4" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG4" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH4" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI4" s="21">
+        <f ca="1">TODAY()+365</f>
+        <v>46190</v>
+      </c>
+      <c r="AJ4" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="AK4" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="AL4" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM4" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="AN4" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="AO4" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="AP4" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="AQ4" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AR4" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS4" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AT4" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU4" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV4" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="AW4" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="AX4" s="27">
+        <v>1234567891</v>
+      </c>
+      <c r="AY4" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AZ4" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="BA4" s="19">
+        <f t="shared" ca="1" si="1"/>
+        <v>45915</v>
+      </c>
+      <c r="BB4" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="BC4" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="BD4" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="BE4" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="BF4" s="19">
+        <f t="shared" ref="BF4:BF7" ca="1" si="5">W4</f>
+        <v>45794</v>
+      </c>
+      <c r="BG4" s="19">
+        <f t="shared" ref="BG4:BG7" ca="1" si="6">W4</f>
+        <v>45794</v>
+      </c>
+      <c r="BH4" s="21">
+        <f t="shared" ref="BH4:BH7" ca="1" si="7">AI4</f>
+        <v>46190</v>
+      </c>
+      <c r="BI4" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BJ4" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="BK4" s="30">
+        <f t="array" aca="1" ref="BK4:BK5" ca="1">_xlfn.RANDARRAY(2,1,123456789,999999999,TRUE)</f>
+        <v>770708346</v>
+      </c>
+      <c r="BL4" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="BM4" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="BN4" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="BO4" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="BP4" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="BQ4" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="BR4" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BS4" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="BT4" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="BU4" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="BV4" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="BW4" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="BX4" s="33"/>
+      <c r="BY4" s="33"/>
+      <c r="BZ4" s="34"/>
+      <c r="CA4" s="34"/>
+      <c r="CB4" s="33"/>
+      <c r="CC4" s="33"/>
+      <c r="CD4" s="33"/>
+      <c r="CE4" s="33"/>
+      <c r="CF4" s="33"/>
+      <c r="CG4" s="33"/>
+      <c r="CH4" s="33"/>
+    </row>
+    <row r="5" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" s="35"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="16"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="L5" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="M5" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="N5" s="18">
+        <v>1</v>
+      </c>
+      <c r="O5" s="18">
+        <v>1612</v>
+      </c>
+      <c r="P5" s="18">
+        <v>90851</v>
+      </c>
+      <c r="Q5" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="R5" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="S5" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="T5" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="U5" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="V5" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="W5" s="21">
+        <f t="shared" ca="1" si="0"/>
+        <v>45794</v>
+      </c>
+      <c r="X5" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y5" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="Z5" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA5" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="AB5" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC5" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="AD5" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE5" s="15">
+        <v>40</v>
+      </c>
+      <c r="AF5" s="23">
+        <v>40</v>
+      </c>
+      <c r="AG5" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH5" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI5" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="AJ5" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="AK5" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="AL5" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="AM5" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="AN5" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="AO5" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="AP5" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="AQ5" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AR5" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS5" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AT5" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU5" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV5" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="AW5" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="AX5" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY5" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AZ5" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="BA5" s="19">
+        <f t="shared" ca="1" si="1"/>
+        <v>45915</v>
+      </c>
+      <c r="BB5" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="BC5" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="BD5" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="BE5" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="BF5" s="19">
+        <f t="shared" ca="1" si="5"/>
+        <v>45794</v>
+      </c>
+      <c r="BG5" s="19">
+        <f t="shared" ca="1" si="6"/>
+        <v>45794</v>
+      </c>
+      <c r="BH5" s="21" t="str">
+        <f t="shared" si="7"/>
+        <v>N/A</v>
+      </c>
+      <c r="BI5" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BJ5" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="BK5" s="30">
+        <f ca="1"/>
+        <v>257672960</v>
+      </c>
+      <c r="BL5" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM5" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="BN5" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="BO5" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="BP5" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="BQ5" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="BR5" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BS5" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="BT5" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="BU5" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="BV5" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="BW5" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="BX5" s="33"/>
+      <c r="BY5" s="33"/>
+      <c r="BZ5" s="34"/>
+      <c r="CA5" s="34"/>
+      <c r="CB5" s="33"/>
+      <c r="CC5" s="33"/>
+      <c r="CD5" s="33"/>
+      <c r="CE5" s="33"/>
+      <c r="CF5" s="33"/>
+      <c r="CG5" s="33"/>
+      <c r="CH5" s="33"/>
+    </row>
+    <row r="6" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="36"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" s="16"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="L6" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="M6" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="N6" s="18">
+        <v>1</v>
+      </c>
+      <c r="O6" s="18">
+        <v>1612</v>
+      </c>
+      <c r="P6" s="18">
+        <v>90851</v>
+      </c>
+      <c r="Q6" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="R6" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="S6" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="T6" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="U6" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="V6" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="W6" s="21">
+        <f t="shared" ca="1" si="0"/>
+        <v>45794</v>
+      </c>
+      <c r="X6" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y6" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="Z6" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA6" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="AB6" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC6" s="15">
+        <v>870</v>
+      </c>
+      <c r="AD6" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE6" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="AF6" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG6" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH6" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI6" s="21">
+        <f ca="1">TODAY()+365</f>
+        <v>46190</v>
+      </c>
+      <c r="AJ6" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="AK6" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="AL6" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="AM6" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="AN6" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="AO6" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="AP6" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="AQ6" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AR6" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS6" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AT6" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU6" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV6" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="AW6" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="AX6" s="27">
+        <v>1234567891</v>
+      </c>
+      <c r="AY6" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AZ6" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="BA6" s="19">
+        <f t="shared" ca="1" si="1"/>
+        <v>45915</v>
+      </c>
+      <c r="BB6" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="BC6" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="BD6" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="BE6" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="BF6" s="19">
+        <f t="shared" ca="1" si="5"/>
+        <v>45794</v>
+      </c>
+      <c r="BG6" s="19">
+        <f t="shared" ca="1" si="6"/>
+        <v>45794</v>
+      </c>
+      <c r="BH6" s="21">
+        <f t="shared" ca="1" si="7"/>
+        <v>46190</v>
+      </c>
+      <c r="BI6" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BJ6" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="BK6" s="30">
+        <f t="array" aca="1" ref="BK6:BK7" ca="1">_xlfn.RANDARRAY(2,1,123456789,999999999,TRUE)</f>
+        <v>223053016</v>
+      </c>
+      <c r="BL6" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="BM6" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="BN6" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="BO6" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="BP6" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="BQ6" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="BR6" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BS6" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="BT6" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="BU6" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="BV6" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="BW6" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="BX6" s="33"/>
+      <c r="BY6" s="33"/>
+      <c r="BZ6" s="34"/>
+      <c r="CA6" s="34"/>
+      <c r="CB6" s="33"/>
+      <c r="CC6" s="33"/>
+      <c r="CD6" s="33"/>
+      <c r="CE6" s="33"/>
+      <c r="CF6" s="33"/>
+      <c r="CG6" s="33"/>
+      <c r="CH6" s="33"/>
+    </row>
+    <row r="7" spans="1:86" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="35"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="16"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="I7" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="J7" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="K7" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="L7" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="M7" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="N7" s="18">
+        <v>1</v>
+      </c>
+      <c r="O7" s="18">
+        <v>1612</v>
+      </c>
+      <c r="P7" s="18">
+        <v>90851</v>
+      </c>
+      <c r="Q7" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="R7" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="S7" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="T7" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="U7" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="V7" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="W7" s="21">
+        <f t="shared" ca="1" si="0"/>
+        <v>45794</v>
+      </c>
+      <c r="X7" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y7" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="Z7" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA7" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="AB7" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC7" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="AD7" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE7" s="15">
+        <v>40</v>
+      </c>
+      <c r="AF7" s="23">
+        <v>40</v>
+      </c>
+      <c r="AG7" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH7" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI7" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="AJ7" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="AK7" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="AL7" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="AM7" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="AN7" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="AO7" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="AP7" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="AQ7" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AR7" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS7" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AT7" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AU7" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="AV7" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="AW7" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="AX7" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="AY7" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="AZ7" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="BA7" s="19">
+        <f t="shared" ca="1" si="1"/>
+        <v>45915</v>
+      </c>
+      <c r="BB7" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="BC7" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="BD7" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="BE7" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="BF7" s="19">
+        <f t="shared" ca="1" si="5"/>
+        <v>45794</v>
+      </c>
+      <c r="BG7" s="19">
+        <f t="shared" ca="1" si="6"/>
+        <v>45794</v>
+      </c>
+      <c r="BH7" s="21" t="str">
+        <f t="shared" si="7"/>
+        <v>N/A</v>
+      </c>
+      <c r="BI7" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BJ7" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="BK7" s="30">
+        <f ca="1"/>
+        <v>671803277</v>
+      </c>
+      <c r="BL7" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM7" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="BN7" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="BO7" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="BP7" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="BQ7" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="BR7" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="BS7" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="BT7" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="BU7" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="BV7" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="BW7" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="BX7" s="33"/>
+      <c r="BY7" s="33"/>
+      <c r="BZ7" s="34"/>
+      <c r="CA7" s="34"/>
+      <c r="CB7" s="33"/>
+      <c r="CC7" s="33"/>
+      <c r="CD7" s="33"/>
+      <c r="CE7" s="33"/>
+      <c r="CF7" s="33"/>
+      <c r="CG7" s="33"/>
+      <c r="CH7" s="33"/>
+    </row>
   </sheetData>
-  <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2:BE3">
-      <formula1>INDIRECT($H2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2:BU3">
-      <formula1>INDIRECT($H2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB3">
-      <formula1>INDIRECT($H2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J3">
-      <formula1>INDIRECT($H2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S3">
-      <formula1>INDIRECT($H2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V3">
-      <formula1>INDIRECT($H2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X3">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2:BE7 X2:X7 V2:V7 S2:S7 J2:J7 CB2:CB7 BU2:BU7" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($H2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="U2" r:id="rId1"/>
-    <hyperlink ref="U3" r:id="rId2"/>
+    <hyperlink ref="U2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="U3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="U4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="U5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="U6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="U7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId7"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>